<commit_message>
Update travel_sheet_v2_approved.xlsx and labeled relocating a column as a noise
</commit_message>
<xml_diff>
--- a/data/travel_sheet_v2_approved.xlsx
+++ b/data/travel_sheet_v2_approved.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arezo-o\Downloads\ArezooHassannezhad\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E661C19E-C5A7-44F5-A6D9-68EA94AB9F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF2459A-205A-4DDE-B2DF-8778DB1325F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -376,7 +376,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -401,6 +401,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -414,12 +420,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -764,7 +771,7 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>